<commit_message>
thêm giải thích đáp án
</commit_message>
<xml_diff>
--- a/question/Question.xlsx
+++ b/question/Question.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\file_luu_tru\du_an\minigame\question\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F6EABAC-A16E-440C-9F9B-F6E02B1457CF}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A0C8BB6-FB23-4F0B-A4E3-301335E38B3B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="17256" windowHeight="5268" xr2:uid="{13D47C2E-6DA5-4663-B107-8F3B884F698D}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="107">
   <si>
     <t>question</t>
   </si>
@@ -138,9 +138,6 @@
     <t>M10</t>
   </si>
   <si>
-    <t>9 cẳng</t>
-  </si>
-  <si>
     <t>sound</t>
   </si>
   <si>
@@ -220,6 +217,148 @@
   </si>
   <si>
     <t>Sai người sai thời điểm</t>
+  </si>
+  <si>
+    <t>explanation</t>
+  </si>
+  <si>
+    <t>explanation_image</t>
+  </si>
+  <si>
+    <t>Ngày 8/3 là Ngày Quốc tế Phụ nữ, tôn vinh phụ nữ trên toàn thế giới.</t>
+  </si>
+  <si>
+    <t>Găng tay vàng trong làng bắt gôn là ??</t>
+  </si>
+  <si>
+    <t>Trương Công Hiện</t>
+  </si>
+  <si>
+    <t>Nguyễn Phương Nguyên</t>
+  </si>
+  <si>
+    <t>Hà Nguyên Vũ</t>
+  </si>
+  <si>
+    <t>Nguyễn Như Quang</t>
+  </si>
+  <si>
+    <t>Phải đọc kĩ nhé. Yêu cầu trả lời ĐÚNG =)))</t>
+  </si>
+  <si>
+    <t>Bà Triệu</t>
+  </si>
+  <si>
+    <t>Hai Bà Trưng</t>
+  </si>
+  <si>
+    <t>Võ Thị Sáu</t>
+  </si>
+  <si>
+    <t>Nguyễn Thị Minh Khai</t>
+  </si>
+  <si>
+    <t>Hai Bà Trưng lãnh đạo cuộc khởi nghĩa năm 40 chống nhà Hán, thể hiện tinh thần anh hùng và vai trò to lớn của phụ nữ Việt Nam trong lịch sử.</t>
+  </si>
+  <si>
+    <t>ngua_cat_dau_moi.jpg</t>
+  </si>
+  <si>
+    <t>Tưởng là ngựa cắt đầu moi không đấy =))))</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Không được nhầm là anh em đâu nhé </t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Câu thành ngữ nào thể hiện </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>tinh thần mạnh mẽ, kiên cường của phụ nữ Việt Nam?</t>
+    </r>
+  </si>
+  <si>
+    <t>Công cha như núi Thái Sơn</t>
+  </si>
+  <si>
+    <t>Giặc đến nhà đàn bà cũng đánh</t>
+  </si>
+  <si>
+    <t>Đèn nhà ai nhà nấy rạng</t>
+  </si>
+  <si>
+    <t>Ăn quả nhớ kẻ trồng cây</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 cây làm chẳng nên non 3 cây chụm lại </t>
+  </si>
+  <si>
+    <t>nên hòn núi cao</t>
+  </si>
+  <si>
+    <t>thì thừa 2 cây</t>
+  </si>
+  <si>
+    <t>vẫn là 3 cây</t>
+  </si>
+  <si>
+    <t>Càng đọc càng thấy tào lao, cây làm nên núi thì tao chết liền</t>
+  </si>
+  <si>
+    <t>Người tính không bằng</t>
+  </si>
+  <si>
+    <t>AI</t>
+  </si>
+  <si>
+    <t>Trời tính</t>
+  </si>
+  <si>
+    <t>Máy tính</t>
+  </si>
+  <si>
+    <t>Có công mài sắt</t>
+  </si>
+  <si>
+    <t>Có ngày nên kim</t>
+  </si>
+  <si>
+    <t>Có ngày tháng năm</t>
+  </si>
+  <si>
+    <t>Có ngày mỏi tay</t>
+  </si>
+  <si>
+    <t>Ngựa ít thôi</t>
+  </si>
+  <si>
+    <t>Đây là câu ???</t>
+  </si>
+  <si>
+    <t>Thắng làm vua thua làm giặc</t>
+  </si>
+  <si>
+    <t>99% con bạc dừng lại trước khi thắng lớn</t>
+  </si>
+  <si>
+    <t>Da màu không mạnh bằng Daden</t>
+  </si>
+  <si>
+    <t>Tốt gỗ hơn tốt nước sơn</t>
+  </si>
+  <si>
+    <t>go_son.mp4</t>
+  </si>
+  <si>
+    <t>Ở Việt Nam, 8/3 còn gắn với cuộc khởi nghĩa nào?</t>
   </si>
 </sst>
 </file>
@@ -263,7 +402,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -274,6 +413,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -588,10 +728,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD6D20C5-F5C4-4FB0-8774-1BDFC45A7A57}">
-  <dimension ref="A1:O51"/>
+  <dimension ref="A1:Q51"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>6</v>
       </c>
@@ -608,7 +748,7 @@
         <v>9</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="G1" s="3" t="s">
         <v>10</v>
@@ -637,8 +777,14 @@
       <c r="O1" s="3" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P1" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="Q1" s="4" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -664,7 +810,7 @@
         <v>16</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="L2" s="1" t="s">
         <v>1</v>
@@ -674,8 +820,11 @@
       </c>
       <c r="N2" s="1"/>
       <c r="O2" s="1"/>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <f>A2+1</f>
         <v>2</v>
@@ -707,7 +856,7 @@
       <c r="N3" s="1"/>
       <c r="O3" s="1"/>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <f t="shared" ref="A4:A51" si="0">A3+1</f>
         <v>3</v>
@@ -719,9 +868,11 @@
         <v>12</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="E4" s="1"/>
+        <v>39</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>78</v>
+      </c>
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
       <c r="H4" s="1" t="s">
@@ -731,7 +882,7 @@
         <v>26</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>37</v>
+        <v>99</v>
       </c>
       <c r="K4" s="1" t="s">
         <v>27</v>
@@ -744,8 +895,11 @@
       </c>
       <c r="N4" s="1"/>
       <c r="O4" s="1"/>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P4" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -777,7 +931,7 @@
       <c r="N5" s="1"/>
       <c r="O5" s="1"/>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -789,19 +943,19 @@
         <v>12</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E6" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="J6" s="1" t="s">
         <v>43</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="I6" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="J6" s="1" t="s">
-        <v>44</v>
       </c>
       <c r="L6" s="1" t="s">
         <v>3</v>
@@ -812,7 +966,7 @@
       <c r="N6" s="1"/>
       <c r="O6" s="1"/>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -824,22 +978,22 @@
         <v>12</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E7" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="H7">
         <v>1</v>
       </c>
       <c r="I7" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="J7" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="K7" t="s">
         <v>49</v>
-      </c>
-      <c r="J7" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="K7" t="s">
-        <v>50</v>
       </c>
       <c r="L7" s="1" t="s">
         <v>1</v>
@@ -849,8 +1003,11 @@
       </c>
       <c r="N7" s="1"/>
       <c r="O7" s="1"/>
-    </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P7" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -862,18 +1019,21 @@
         <v>17</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="L8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="M8" s="2">
         <v>5</v>
       </c>
       <c r="N8" s="1"/>
       <c r="O8" s="1"/>
-    </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P8" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -885,22 +1045,22 @@
         <v>12</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G9" t="s">
+        <v>52</v>
+      </c>
+      <c r="H9" t="s">
         <v>53</v>
       </c>
-      <c r="H9" t="s">
+      <c r="I9" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="I9" s="1" t="s">
+      <c r="J9" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="K9" t="s">
         <v>55</v>
-      </c>
-      <c r="J9" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="K9" t="s">
-        <v>56</v>
       </c>
       <c r="L9" s="1" t="s">
         <v>2</v>
@@ -911,7 +1071,7 @@
       <c r="N9" s="1"/>
       <c r="O9" s="1"/>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <f t="shared" si="0"/>
         <v>9</v>
@@ -923,22 +1083,22 @@
         <v>12</v>
       </c>
       <c r="D10" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="F10" t="s">
+        <v>58</v>
+      </c>
+      <c r="H10" t="s">
         <v>60</v>
       </c>
-      <c r="F10" t="s">
-        <v>59</v>
-      </c>
-      <c r="H10" t="s">
+      <c r="I10" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="I10" s="1" t="s">
+      <c r="J10" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="J10" s="1" t="s">
+      <c r="K10" t="s">
         <v>63</v>
-      </c>
-      <c r="K10" t="s">
-        <v>64</v>
       </c>
       <c r="L10" s="1" t="s">
         <v>1</v>
@@ -949,7 +1109,7 @@
       <c r="N10" s="1"/>
       <c r="O10" s="1"/>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -960,13 +1120,34 @@
       <c r="C11" s="1" t="s">
         <v>12</v>
       </c>
+      <c r="D11" t="s">
+        <v>106</v>
+      </c>
+      <c r="H11" t="s">
+        <v>73</v>
+      </c>
+      <c r="I11" t="s">
+        <v>74</v>
+      </c>
+      <c r="J11" t="s">
+        <v>75</v>
+      </c>
+      <c r="K11" t="s">
+        <v>76</v>
+      </c>
+      <c r="L11" t="s">
+        <v>2</v>
+      </c>
       <c r="M11" s="2">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="N11" s="1"/>
       <c r="O11" s="1"/>
-    </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P11" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -977,13 +1158,31 @@
       <c r="C12" s="1" t="s">
         <v>12</v>
       </c>
+      <c r="D12" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="H12" t="s">
+        <v>88</v>
+      </c>
+      <c r="I12" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="J12" t="s">
+        <v>87</v>
+      </c>
+      <c r="L12" s="1" t="s">
+        <v>3</v>
+      </c>
       <c r="M12" s="2">
         <v>5</v>
       </c>
       <c r="N12" s="1"/>
       <c r="O12" s="1"/>
-    </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P12" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -994,13 +1193,28 @@
       <c r="C13" s="1" t="s">
         <v>12</v>
       </c>
+      <c r="D13" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="H13" t="s">
+        <v>92</v>
+      </c>
+      <c r="I13" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="J13" t="s">
+        <v>94</v>
+      </c>
+      <c r="L13" s="1" t="s">
+        <v>2</v>
+      </c>
       <c r="M13" s="2">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="N13" s="1"/>
       <c r="O13" s="1"/>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A14" s="1">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -1011,13 +1225,28 @@
       <c r="C14" s="1" t="s">
         <v>12</v>
       </c>
+      <c r="D14" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="H14" t="s">
+        <v>96</v>
+      </c>
+      <c r="I14" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="J14" t="s">
+        <v>98</v>
+      </c>
+      <c r="L14" s="1" t="s">
+        <v>1</v>
+      </c>
       <c r="M14" s="2">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="N14" s="1"/>
       <c r="O14" s="1"/>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A15" s="1">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -1028,11 +1257,32 @@
       <c r="C15" s="1" t="s">
         <v>12</v>
       </c>
+      <c r="D15" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="G15" t="s">
+        <v>105</v>
+      </c>
+      <c r="H15" t="s">
+        <v>101</v>
+      </c>
+      <c r="I15" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="J15" t="s">
+        <v>103</v>
+      </c>
+      <c r="K15" t="s">
+        <v>104</v>
+      </c>
+      <c r="L15" s="1" t="s">
+        <v>4</v>
+      </c>
       <c r="M15" s="2">
         <v>10</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A16" s="1">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -1043,6 +1293,24 @@
       <c r="C16" s="1" t="s">
         <v>12</v>
       </c>
+      <c r="D16" t="s">
+        <v>81</v>
+      </c>
+      <c r="H16" t="s">
+        <v>82</v>
+      </c>
+      <c r="I16" t="s">
+        <v>83</v>
+      </c>
+      <c r="J16" t="s">
+        <v>84</v>
+      </c>
+      <c r="K16" t="s">
+        <v>85</v>
+      </c>
+      <c r="L16" t="s">
+        <v>2</v>
+      </c>
       <c r="M16" s="2">
         <v>10</v>
       </c>
@@ -1436,12 +1704,6 @@
       <c r="M42" s="2">
         <v>0</v>
       </c>
-      <c r="N42">
-        <v>10</v>
-      </c>
-      <c r="O42">
-        <v>20</v>
-      </c>
     </row>
     <row r="43" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A43" s="1">
@@ -1508,8 +1770,32 @@
       <c r="C45" s="1" t="s">
         <v>12</v>
       </c>
+      <c r="D45" t="s">
+        <v>67</v>
+      </c>
+      <c r="H45" t="s">
+        <v>68</v>
+      </c>
+      <c r="I45" t="s">
+        <v>69</v>
+      </c>
+      <c r="J45" t="s">
+        <v>70</v>
+      </c>
+      <c r="K45" t="s">
+        <v>71</v>
+      </c>
+      <c r="L45" t="s">
+        <v>4</v>
+      </c>
       <c r="M45" s="2">
         <v>0</v>
+      </c>
+      <c r="N45">
+        <v>10</v>
+      </c>
+      <c r="O45">
+        <v>15</v>
       </c>
     </row>
     <row r="46" spans="1:15" x14ac:dyDescent="0.3">

</xml_diff>